<commit_message>
Automate GitHub Actions database ingestion: write directly to data/standings_latest.json, auto-export CSV/Excel, and commit to repo
</commit_message>
<xml_diff>
--- a/exports/motorsport_database_2026.xlsx
+++ b/exports/motorsport_database_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea\Desktop\Sito overrevving\exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9237B815-A676-4E57-BF82-5A3528EA71E1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2FBFB2C-0B38-4D79-95A3-7B2104A612A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="19845" xr2:uid="{8B68D311-E33E-4B19-A776-84924D22BFC1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51600" windowHeight="19845" xr2:uid="{585B7A87-0D47-4F02-AC92-C924EEA56768}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendars_2026" sheetId="4" r:id="rId1"/>
@@ -1515,7 +1515,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D4C9B0E-8C47-4EE8-B71C-D2C006BE7F33}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8BB0742-D075-4779-855A-66CF89C10A7D}">
   <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4253,7 +4253,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613CFA2D-DB22-4CC9-8B63-265364522DB4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09D99BF9-5EDC-4508-928D-EBA176CC3AD1}">
   <dimension ref="A1:M1553"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -67951,7 +67951,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8248567D-F1D0-46DF-971B-04CEF7B38058}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{740E35D8-84AE-4C01-B0AB-485CFD4DC6C8}">
   <dimension ref="A1:H302"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>